<commit_message>
Add v19 segment workbench, parent allocation report, trading plan + multi-source BTC fetcher
- code/update_btc_price_fred.py: add Yahoo + Coinbase fallbacks so daily
  data stays current when FRED lags (FRED -> append Yahoo newer rows ->
  Coinbase recent candles, with local-file fallback path)
- data: refresh btc_price_fred + btc_merged_daily through latest
- analysis_runs/2026-06-04_segment_experiments: v19 segment-cycle
  workbench (py/html), case ledger, saved samples + summaries, runbook
- analysis_runs/2026-06-07_parent_btc_allocation_report: parent-facing
  2026 allocation report (md/html/pdf/txt), AHR999 cycle overlay,
  on-chain + peak-structure charts
- trading_plan_2026_2030.md: next-cycle buy/sell discipline plan
- visualization/2026-06-05: stepA3 pre-data summary
- .gitignore: ignore *.log (server runtime logs)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/btc_merged_daily.xlsx
+++ b/data/btc_merged_daily.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4201"/>
+  <dimension ref="A1:C4206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55049,6 +55049,71 @@
         </is>
       </c>
     </row>
+    <row r="4202">
+      <c r="A4202" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B4202" t="n">
+        <v>71319.7734375</v>
+      </c>
+      <c r="C4202" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4203">
+      <c r="A4203" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B4203" t="n">
+        <v>66703.65625</v>
+      </c>
+      <c r="C4203" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4204">
+      <c r="A4204" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B4204" t="n">
+        <v>64014.3671875</v>
+      </c>
+      <c r="C4204" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4205">
+      <c r="A4205" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B4205" t="n">
+        <v>63801.57421875</v>
+      </c>
+      <c r="C4205" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4206">
+      <c r="A4206" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B4206" t="n">
+        <v>60714.25</v>
+      </c>
+      <c r="C4206" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh BTC data to 2026-07-17; add 06-25 + 07-17 parent report versions
- data: BTC merged/FRED updated through 2026-07-17 (bounced to $63,932 / AHR 0.339 after a 06-30 low of $58,366 / 0.279)
- parent allocation report: new dated versions 2026-06-25 (deep-value) and 2026-07-17 (W-bottom bounce), each md/html/pdf/txt
- regenerate AHR999 cycle overlay + peak-structure + real-user charts to latest
- §5 on-chain refreshed to June via web (LTH switched to Glassnode 14.12M->14.8M, ETF/treasury updated); lth_metrics.csv now Glassnode-consistent
- visualization: stepA3 summaries for 2026-06-25 / 06-30 / 07-17

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/btc_merged_daily.xlsx
+++ b/data/btc_merged_daily.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4206"/>
+  <dimension ref="A1:C4248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55054,7 +55054,7 @@
         <v>46174</v>
       </c>
       <c r="B4202" t="n">
-        <v>71319.7734375</v>
+        <v>71263.63</v>
       </c>
       <c r="C4202" t="inlineStr">
         <is>
@@ -55067,7 +55067,7 @@
         <v>46175</v>
       </c>
       <c r="B4203" t="n">
-        <v>66703.65625</v>
+        <v>66661.02</v>
       </c>
       <c r="C4203" t="inlineStr">
         <is>
@@ -55080,7 +55080,7 @@
         <v>46176</v>
       </c>
       <c r="B4204" t="n">
-        <v>64014.3671875</v>
+        <v>64257.19</v>
       </c>
       <c r="C4204" t="inlineStr">
         <is>
@@ -55093,7 +55093,7 @@
         <v>46177</v>
       </c>
       <c r="B4205" t="n">
-        <v>63801.57421875</v>
+        <v>63742.66</v>
       </c>
       <c r="C4205" t="inlineStr">
         <is>
@@ -55106,9 +55106,555 @@
         <v>46178</v>
       </c>
       <c r="B4206" t="n">
-        <v>60714.25</v>
+        <v>61272.32</v>
       </c>
       <c r="C4206" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4207">
+      <c r="A4207" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B4207" t="n">
+        <v>60881.64</v>
+      </c>
+      <c r="C4207" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4208">
+      <c r="A4208" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B4208" t="n">
+        <v>63216.78</v>
+      </c>
+      <c r="C4208" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4209">
+      <c r="A4209" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B4209" t="n">
+        <v>63049.86</v>
+      </c>
+      <c r="C4209" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4210">
+      <c r="A4210" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B4210" t="n">
+        <v>61751.94</v>
+      </c>
+      <c r="C4210" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4211">
+      <c r="A4211" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B4211" t="n">
+        <v>61570.02</v>
+      </c>
+      <c r="C4211" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4212">
+      <c r="A4212" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B4212" t="n">
+        <v>63482.72</v>
+      </c>
+      <c r="C4212" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4213">
+      <c r="A4213" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B4213" t="n">
+        <v>63554.96</v>
+      </c>
+      <c r="C4213" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4214">
+      <c r="A4214" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B4214" t="n">
+        <v>64374.02</v>
+      </c>
+      <c r="C4214" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4215">
+      <c r="A4215" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B4215" t="n">
+        <v>65605.03999999999</v>
+      </c>
+      <c r="C4215" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4216">
+      <c r="A4216" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B4216" t="n">
+        <v>66231.94</v>
+      </c>
+      <c r="C4216" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4217">
+      <c r="A4217" s="2" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B4217" t="n">
+        <v>65679.13</v>
+      </c>
+      <c r="C4217" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4218">
+      <c r="A4218" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B4218" t="n">
+        <v>64529.96</v>
+      </c>
+      <c r="C4218" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4219">
+      <c r="A4219" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B4219" t="n">
+        <v>62852.71</v>
+      </c>
+      <c r="C4219" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4220">
+      <c r="A4220" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B4220" t="n">
+        <v>63522.76</v>
+      </c>
+      <c r="C4220" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4221">
+      <c r="A4221" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B4221" t="n">
+        <v>64180</v>
+      </c>
+      <c r="C4221" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4222">
+      <c r="A4222" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B4222" t="n">
+        <v>63321.17</v>
+      </c>
+      <c r="C4222" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4223">
+      <c r="A4223" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B4223" t="n">
+        <v>63932.91</v>
+      </c>
+      <c r="C4223" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4224">
+      <c r="A4224" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B4224" t="n">
+        <v>62689.99</v>
+      </c>
+      <c r="C4224" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4225">
+      <c r="A4225" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B4225" t="n">
+        <v>60950</v>
+      </c>
+      <c r="C4225" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4226">
+      <c r="A4226" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B4226" t="n">
+        <v>59778.75</v>
+      </c>
+      <c r="C4226" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4227">
+      <c r="A4227" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B4227" t="n">
+        <v>59995.84</v>
+      </c>
+      <c r="C4227" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4228">
+      <c r="A4228" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B4228" t="n">
+        <v>59964.66</v>
+      </c>
+      <c r="C4228" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4229">
+      <c r="A4229" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B4229" t="n">
+        <v>59367.05</v>
+      </c>
+      <c r="C4229" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4230">
+      <c r="A4230" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B4230" t="n">
+        <v>60128.09</v>
+      </c>
+      <c r="C4230" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4231">
+      <c r="A4231" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4231" t="n">
+        <v>58585.96</v>
+      </c>
+      <c r="C4231" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4232">
+      <c r="A4232" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4232" t="n">
+        <v>59881.98</v>
+      </c>
+      <c r="C4232" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4233">
+      <c r="A4233" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4233" t="n">
+        <v>61422.31</v>
+      </c>
+      <c r="C4233" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4234">
+      <c r="A4234" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B4234" t="n">
+        <v>62537.99</v>
+      </c>
+      <c r="C4234" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4235">
+      <c r="A4235" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B4235" t="n">
+        <v>63027.09</v>
+      </c>
+      <c r="C4235" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4236">
+      <c r="A4236" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B4236" t="n">
+        <v>63577.07</v>
+      </c>
+      <c r="C4236" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4237">
+      <c r="A4237" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B4237" t="n">
+        <v>63980.01</v>
+      </c>
+      <c r="C4237" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4238">
+      <c r="A4238" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B4238" t="n">
+        <v>63367.99</v>
+      </c>
+      <c r="C4238" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4239">
+      <c r="A4239" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B4239" t="n">
+        <v>62168.43</v>
+      </c>
+      <c r="C4239" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4240">
+      <c r="A4240" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B4240" t="n">
+        <v>63156.18</v>
+      </c>
+      <c r="C4240" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4241">
+      <c r="A4241" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B4241" t="n">
+        <v>64057.01</v>
+      </c>
+      <c r="C4241" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4242">
+      <c r="A4242" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B4242" t="n">
+        <v>63831.03</v>
+      </c>
+      <c r="C4242" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4243">
+      <c r="A4243" s="2" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B4243" t="n">
+        <v>63809.21</v>
+      </c>
+      <c r="C4243" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4244">
+      <c r="A4244" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B4244" t="n">
+        <v>62233.29</v>
+      </c>
+      <c r="C4244" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4245">
+      <c r="A4245" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B4245" t="n">
+        <v>64967.74</v>
+      </c>
+      <c r="C4245" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4246">
+      <c r="A4246" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B4246" t="n">
+        <v>64755.57</v>
+      </c>
+      <c r="C4246" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4247">
+      <c r="A4247" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B4247" t="n">
+        <v>63746.78</v>
+      </c>
+      <c r="C4247" t="inlineStr">
+        <is>
+          <t>btc_price_fred</t>
+        </is>
+      </c>
+    </row>
+    <row r="4248">
+      <c r="A4248" s="2" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B4248" t="n">
+        <v>63931.55078125</v>
+      </c>
+      <c r="C4248" t="inlineStr">
         <is>
           <t>btc_price_fred</t>
         </is>

</xml_diff>